<commit_message>
v511: template Stock Asig - banda BACKORDER + rows altura 40 + autofilter PEDIDO
Cambios en templates/stock_asig_template.xlsx:
- Banda BACKORDER: merge F1:H4 con texto 'BACKORDER' 48pt bold
  centrado sobre fondo celeste #00A9E0. Reemplaza el logo Shimano
  embebido (drawing eliminado del xlsx).
- Fondo celeste #B3E5FA para toda la banda superior filas 1-2 col
  A-J (excepto donde ya hay contenido). Filas 1-4 con altura 32px.
- CLIENTE + CUIT labels con fondo gris #D0D0D0 y bold.

Cambios en _buildStockAsigBufferConTemplate:
- Cada row de producto ahora tiene row.height = 40 + wrap text +
  vertical middle (matchea la row 58 del ejemplo user). Descripcion
  con horizontal left; el resto horizontal center.
- Autofilter con custom filter en columna I (PEDIDO):
  customFilters: [{val: ' ', operator: 'greaterThan'}] - excluye
  celdas vacias. Al abrir el Excel se ven solo los SKUs con qty
  asignada; los otros filtros quedan disponibles sin criterio.
</commit_message>
<xml_diff>
--- a/templates/stock_asig_template.xlsx
+++ b/templates/stock_asig_template.xlsx
@@ -21,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-[$ARS]\ * #,##0_-;\-[$ARS]\ * #,##0_-;_-[$ARS]\ * &quot;-&quot;_-;_-@_-"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -154,8 +154,19 @@
       <sz val="10"/>
       <scheme val="minor"/>
     </font>
+    <font/>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="48"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -196,6 +207,24 @@
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0000A9E0"/>
+        <bgColor rgb="0000A9E0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B3E5FA"/>
+        <bgColor rgb="00B3E5FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D0D0D0"/>
+        <bgColor rgb="00D0D0D0"/>
       </patternFill>
     </fill>
   </fills>
@@ -272,7 +301,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center"/>
@@ -415,6 +444,31 @@
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="18" fillId="9" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="1">
       <protection locked="0" hidden="0"/>
     </xf>
   </cellXfs>
@@ -1034,7 +1088,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="12"/>
   <cols>
     <col width="12.453125" customWidth="1" style="7" min="1" max="1"/>
@@ -1050,51 +1104,51 @@
     <col width="11.453125" customWidth="1" style="2" min="11" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" ht="27.5" customHeight="1">
-      <c r="A1" s="34" t="inlineStr">
-        <is>
-          <t>VER CATALOGO SHIMANO</t>
-        </is>
-      </c>
-      <c r="B1" s="39" t="n"/>
-      <c r="C1" s="39" t="n"/>
-      <c r="D1" s="39" t="n"/>
-      <c r="E1" s="39" t="n"/>
-      <c r="F1" s="37" t="e">
-        <v>#VALUE!</v>
-      </c>
-      <c r="G1" s="39" t="n"/>
-      <c r="H1" s="39" t="n"/>
-      <c r="I1" s="36" t="inlineStr">
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="42" t="n"/>
+      <c r="B1" s="43" t="n"/>
+      <c r="C1" s="43" t="n"/>
+      <c r="D1" s="43" t="n"/>
+      <c r="E1" s="43" t="n"/>
+      <c r="F1" s="44" t="inlineStr">
+        <is>
+          <t>BACKORDER</t>
+        </is>
+      </c>
+      <c r="G1" s="45" t="n"/>
+      <c r="H1" s="45" t="n"/>
+      <c r="I1" s="42" t="inlineStr">
         <is>
           <t>Total Pedido</t>
         </is>
       </c>
-      <c r="J1" s="39" t="n"/>
+      <c r="J1" s="45" t="n"/>
+      <c r="K1" s="46" t="n"/>
     </row>
-    <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="39" t="n"/>
-      <c r="B2" s="39" t="n"/>
-      <c r="C2" s="39" t="n"/>
-      <c r="D2" s="39" t="n"/>
-      <c r="E2" s="39" t="n"/>
-      <c r="F2" s="39" t="n"/>
-      <c r="G2" s="39" t="n"/>
-      <c r="H2" s="39" t="n"/>
-      <c r="I2" s="35">
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="43" t="n"/>
+      <c r="B2" s="43" t="n"/>
+      <c r="C2" s="43" t="n"/>
+      <c r="D2" s="43" t="n"/>
+      <c r="E2" s="43" t="n"/>
+      <c r="F2" s="45" t="n"/>
+      <c r="G2" s="45" t="n"/>
+      <c r="H2" s="45" t="n"/>
+      <c r="I2" s="47">
         <f>SUM(J6:J1005)</f>
         <v/>
       </c>
-      <c r="J2" s="39" t="n"/>
+      <c r="J2" s="45" t="n"/>
+      <c r="K2" s="46" t="n"/>
     </row>
-    <row r="3" ht="14.5" customHeight="1">
-      <c r="A3" s="33" t="inlineStr">
+    <row r="3" ht="32" customHeight="1">
+      <c r="A3" s="48" t="inlineStr">
         <is>
           <t>CLIENTE</t>
         </is>
       </c>
       <c r="B3" s="40" t="n"/>
-      <c r="C3" s="38" t="inlineStr"/>
+      <c r="C3" s="49" t="n"/>
       <c r="D3" s="41" t="n"/>
       <c r="E3" s="40" t="n"/>
       <c r="F3" s="39" t="n"/>
@@ -1102,22 +1156,24 @@
       <c r="H3" s="39" t="n"/>
       <c r="I3" s="39" t="n"/>
       <c r="J3" s="39" t="n"/>
+      <c r="K3" s="46" t="n"/>
     </row>
-    <row r="4" ht="14.5" customHeight="1">
-      <c r="A4" s="33" t="inlineStr">
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="48" t="inlineStr">
         <is>
           <t>CUIT</t>
         </is>
       </c>
       <c r="B4" s="40" t="n"/>
-      <c r="C4" s="38" t="inlineStr"/>
+      <c r="C4" s="49" t="n"/>
       <c r="D4" s="41" t="n"/>
       <c r="E4" s="40" t="n"/>
       <c r="F4" s="39" t="n"/>
       <c r="G4" s="39" t="n"/>
       <c r="H4" s="39" t="n"/>
-      <c r="I4" s="37" t="n"/>
-      <c r="J4" s="37" t="n"/>
+      <c r="I4" s="50" t="n"/>
+      <c r="J4" s="50" t="n"/>
+      <c r="K4" s="46" t="n"/>
     </row>
     <row r="5" ht="32.5" customFormat="1" customHeight="1" s="4">
       <c r="A5" s="3" t="inlineStr">
@@ -1867,13 +1923,12 @@
       </customFilters>
     </filterColumn>
   </autoFilter>
-  <mergeCells count="8">
+  <mergeCells count="7">
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="F1:H4"/>
     <mergeCell ref="I2:J3"/>
     <mergeCell ref="C4:E4"/>
     <mergeCell ref="C3:E3"/>
-    <mergeCell ref="A1:E2"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="I1:J1"/>
   </mergeCells>
@@ -1967,7 +2022,6 @@
           <t>Nombre del transporte</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr"/>
     </row>
     <row r="2" ht="51" customFormat="1" customHeight="1" s="25">
       <c r="A2" s="26" t="inlineStr">
@@ -1975,7 +2029,6 @@
           <t>Domicilio de Entrega (dirección, localidad)</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3" ht="52" customFormat="1" customHeight="1" s="25">
       <c r="A3" s="26" t="inlineStr">
@@ -1983,7 +2036,6 @@
           <t>Domicilio comercial (final cliente)</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
     </row>
     <row r="4" ht="60" customFormat="1" customHeight="1" s="25">
       <c r="A4" s="27" t="inlineStr">
@@ -1991,7 +2043,6 @@
           <t>Teléfono</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
     </row>
     <row r="5" ht="60" customFormat="1" customHeight="1" s="25">
       <c r="A5" s="27" t="inlineStr">
@@ -1999,7 +2050,6 @@
           <t>Horario de Recepción</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
     </row>
     <row r="6" ht="73" customFormat="1" customHeight="1" s="25">
       <c r="A6" s="27" t="inlineStr">
@@ -2007,7 +2057,6 @@
           <t>Contacto</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
     </row>
     <row r="7" ht="23" customFormat="1" customHeight="1" s="25">
       <c r="A7" s="27" t="inlineStr">
@@ -2015,7 +2064,6 @@
           <t>Vendedores</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
     </row>
     <row r="8" ht="20.5" customFormat="1" customHeight="1" s="25">
       <c r="A8" s="27" t="inlineStr">
@@ -2023,7 +2071,6 @@
           <t>Método de Pago</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
     </row>
     <row r="9" ht="24" customFormat="1" customHeight="1" s="31">
       <c r="A9" s="27" t="inlineStr">

</xml_diff>